<commit_message>
chore(templates): update demo Excel templates
Replace 不提取 and 提取 template workbooks in root and BX/IRR and SI/templates for download and local use.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/BX/IRR and SI/templates/不提取模板.xlsx
+++ b/BX/IRR and SI/templates/不提取模板.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\N-21AJPF46TWSF-Data\chenwang\Desktop\my cursor\BX\IRR and SI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3940BB0-CD18-4C59-9577-FBB8CFFC2B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF733B7-1920-494E-B749-2AF2147F670B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="储蓄利益演示" sheetId="1" r:id="rId1"/>
@@ -28,598 +28,298 @@
     <t>預期總現價</t>
   </si>
   <si>
-    <t>1年/21歲</t>
-  </si>
-  <si>
-    <t>2年/22歲</t>
-  </si>
-  <si>
     <t>9,000</t>
   </si>
   <si>
-    <t>3年/23歲</t>
-  </si>
-  <si>
     <t>21,735</t>
   </si>
   <si>
-    <t>4年/24歲</t>
-  </si>
-  <si>
     <t>36,273</t>
   </si>
   <si>
-    <t>5年/25歲</t>
-  </si>
-  <si>
     <t>61,188</t>
   </si>
   <si>
-    <t>6年/26歲</t>
-  </si>
-  <si>
     <t>100,013</t>
   </si>
   <si>
-    <t>7年/27歲</t>
-  </si>
-  <si>
     <t>111,584</t>
   </si>
   <si>
-    <t>8年/28歲</t>
-  </si>
-  <si>
     <t>124,120</t>
   </si>
   <si>
-    <t>9年/29歲</t>
-  </si>
-  <si>
     <t>132,637</t>
   </si>
   <si>
-    <t>10年/30歲</t>
-  </si>
-  <si>
     <t>140,140</t>
   </si>
   <si>
-    <t>11年/31歲</t>
-  </si>
-  <si>
     <t>158,980</t>
   </si>
   <si>
-    <t>12年/32歲</t>
-  </si>
-  <si>
     <t>172,212</t>
   </si>
   <si>
-    <t>13年/33歲</t>
-  </si>
-  <si>
     <t>187,350</t>
   </si>
   <si>
-    <t>14年/34歲</t>
-  </si>
-  <si>
     <t>198,399</t>
   </si>
   <si>
-    <t>15年/35歲</t>
-  </si>
-  <si>
     <t>210,451</t>
   </si>
   <si>
-    <t>16年/36歲</t>
-  </si>
-  <si>
     <t>222,813</t>
   </si>
   <si>
-    <t>17年/37歲</t>
-  </si>
-  <si>
     <t>236,797</t>
   </si>
   <si>
-    <t>18年/38歲</t>
-  </si>
-  <si>
     <t>252,218</t>
   </si>
   <si>
-    <t>19年/39歲</t>
-  </si>
-  <si>
     <t>269,717</t>
   </si>
   <si>
-    <t>20年/40歲</t>
-  </si>
-  <si>
     <t>286,410</t>
   </si>
   <si>
-    <t>21年/41歲</t>
-  </si>
-  <si>
     <t>303,610</t>
   </si>
   <si>
-    <t>22年/42歲</t>
-  </si>
-  <si>
     <t>321,841</t>
   </si>
   <si>
-    <t>23年/43歲</t>
-  </si>
-  <si>
     <t>341,167</t>
   </si>
   <si>
-    <t>24年/44歲</t>
-  </si>
-  <si>
     <t>361,714</t>
   </si>
   <si>
-    <t>25年/45歲</t>
-  </si>
-  <si>
     <t>383,435</t>
   </si>
   <si>
-    <t>26年/46歲</t>
-  </si>
-  <si>
     <t>406,489</t>
   </si>
   <si>
-    <t>27年/47歲</t>
-  </si>
-  <si>
     <t>430,969</t>
   </si>
   <si>
-    <t>28年/48歲</t>
-  </si>
-  <si>
     <t>458,166</t>
   </si>
   <si>
-    <t>29年/49歲</t>
-  </si>
-  <si>
     <t>488,512</t>
   </si>
   <si>
-    <t>30年/50歲</t>
-  </si>
-  <si>
     <t>521,349</t>
   </si>
   <si>
-    <t>31年/51歲</t>
-  </si>
-  <si>
     <t>556,678</t>
   </si>
   <si>
-    <t>32年/52歲</t>
-  </si>
-  <si>
     <t>594,897</t>
   </si>
   <si>
-    <t>33年/53歲</t>
-  </si>
-  <si>
     <t>636,246</t>
   </si>
   <si>
-    <t>34年/54歲</t>
-  </si>
-  <si>
     <t>680,724</t>
   </si>
   <si>
-    <t>35年/55歲</t>
-  </si>
-  <si>
     <t>728,832</t>
   </si>
   <si>
-    <t>36年/56歲</t>
-  </si>
-  <si>
     <t>780,868</t>
   </si>
   <si>
-    <t>37年/57歲</t>
-  </si>
-  <si>
     <t>837,159</t>
   </si>
   <si>
-    <t>38年/58歲</t>
-  </si>
-  <si>
     <t>898,056</t>
   </si>
   <si>
-    <t>39年/59歲</t>
-  </si>
-  <si>
     <t>963,554</t>
   </si>
   <si>
-    <t>40年/60歲</t>
-  </si>
-  <si>
     <t>1,034,389</t>
   </si>
   <si>
-    <t>41年/61歲</t>
-  </si>
-  <si>
     <t>1,111,750</t>
   </si>
   <si>
-    <t>42年/62歲</t>
-  </si>
-  <si>
     <t>1,195,425</t>
   </si>
   <si>
-    <t>43年/63歲</t>
-  </si>
-  <si>
     <t>1,285,933</t>
   </si>
   <si>
-    <t>44年/64歲</t>
-  </si>
-  <si>
     <t>1,383,257</t>
   </si>
   <si>
-    <t>45年/65歲</t>
-  </si>
-  <si>
     <t>1,488,491</t>
   </si>
   <si>
-    <t>46年/66歲</t>
-  </si>
-  <si>
     <t>1,602,280</t>
   </si>
   <si>
-    <t>47年/67歲</t>
-  </si>
-  <si>
     <t>1,707,864</t>
   </si>
   <si>
-    <t>48年/68歲</t>
-  </si>
-  <si>
     <t>1,818,875</t>
   </si>
   <si>
-    <t>49年/69歲</t>
-  </si>
-  <si>
     <t>1,937,102</t>
   </si>
   <si>
-    <t>50年/70歲</t>
-  </si>
-  <si>
     <t>2,063,013</t>
   </si>
   <si>
-    <t>51年/71歲</t>
-  </si>
-  <si>
     <t>2,197,109</t>
   </si>
   <si>
-    <t>52年/72歲</t>
-  </si>
-  <si>
     <t>2,339,921</t>
   </si>
   <si>
-    <t>53年/73歲</t>
-  </si>
-  <si>
     <t>2,492,016</t>
   </si>
   <si>
-    <t>54年/74歲</t>
-  </si>
-  <si>
     <t>2,653,997</t>
   </si>
   <si>
-    <t>55年/75歲</t>
-  </si>
-  <si>
     <t>2,826,507</t>
   </si>
   <si>
-    <t>56年/76歲</t>
-  </si>
-  <si>
     <t>3,010,230</t>
   </si>
   <si>
-    <t>57年/77歲</t>
-  </si>
-  <si>
     <t>3,205,895</t>
   </si>
   <si>
-    <t>58年/78歲</t>
-  </si>
-  <si>
     <t>3,414,278</t>
   </si>
   <si>
-    <t>59年/79歲</t>
-  </si>
-  <si>
     <t>3,636,206</t>
   </si>
   <si>
-    <t>60年/80歲</t>
-  </si>
-  <si>
     <t>3,872,560</t>
   </si>
   <si>
-    <t>61年/81歲</t>
-  </si>
-  <si>
     <t>4,124,276</t>
   </si>
   <si>
-    <t>62年/82歲</t>
-  </si>
-  <si>
     <t>4,392,354</t>
   </si>
   <si>
-    <t>63年/83歲</t>
-  </si>
-  <si>
     <t>4,677,857</t>
   </si>
   <si>
-    <t>64年/84歲</t>
-  </si>
-  <si>
     <t>4,981,918</t>
   </si>
   <si>
-    <t>65年/85歲</t>
-  </si>
-  <si>
     <t>5,305,742</t>
   </si>
   <si>
-    <t>66年/86歲</t>
-  </si>
-  <si>
     <t>5,650,615</t>
   </si>
   <si>
-    <t>67年/87歲</t>
-  </si>
-  <si>
     <t>6,017,905</t>
   </si>
   <si>
-    <t>68年/88歲</t>
-  </si>
-  <si>
     <t>6,409,069</t>
   </si>
   <si>
-    <t>69年/89歲</t>
-  </si>
-  <si>
     <t>6,825,659</t>
   </si>
   <si>
-    <t>70年/90歲</t>
-  </si>
-  <si>
     <t>7,269,327</t>
   </si>
   <si>
-    <t>71年/91歲</t>
-  </si>
-  <si>
     <t>7,741,833</t>
   </si>
   <si>
-    <t>72年/92歲</t>
-  </si>
-  <si>
     <t>8,245,052</t>
   </si>
   <si>
-    <t>73年/93歲</t>
-  </si>
-  <si>
     <t>8,780,980</t>
   </si>
   <si>
-    <t>74年/94歲</t>
-  </si>
-  <si>
     <t>9,351,744</t>
   </si>
   <si>
-    <t>75年/95歲</t>
-  </si>
-  <si>
     <t>9,959,608</t>
   </si>
   <si>
-    <t>76年/96歲</t>
-  </si>
-  <si>
     <t>10,606,982</t>
   </si>
   <si>
-    <t>77年/97歲</t>
-  </si>
-  <si>
     <t>11,296,436</t>
   </si>
   <si>
-    <t>78年/98歲</t>
-  </si>
-  <si>
     <t>12,030,704</t>
   </si>
   <si>
-    <t>79年/99歲</t>
-  </si>
-  <si>
     <t>12,812,700</t>
   </si>
   <si>
-    <t>80年/100歲</t>
-  </si>
-  <si>
     <t>13,645,525</t>
   </si>
   <si>
-    <t>81年/101歲</t>
-  </si>
-  <si>
     <t>14,532,485</t>
   </si>
   <si>
-    <t>82年/102歲</t>
-  </si>
-  <si>
     <t>15,477,096</t>
   </si>
   <si>
-    <t>83年/103歲</t>
-  </si>
-  <si>
     <t>16,483,107</t>
   </si>
   <si>
-    <t>84年/104歲</t>
-  </si>
-  <si>
     <t>17,554,509</t>
   </si>
   <si>
-    <t>85年/105歲</t>
-  </si>
-  <si>
     <t>18,695,552</t>
   </si>
   <si>
-    <t>86年/106歲</t>
-  </si>
-  <si>
     <t>19,910,763</t>
   </si>
   <si>
-    <t>87年/107歲</t>
-  </si>
-  <si>
     <t>21,204,963</t>
   </si>
   <si>
-    <t>88年/108歲</t>
-  </si>
-  <si>
     <t>22,583,286</t>
   </si>
   <si>
-    <t>89年/109歲</t>
-  </si>
-  <si>
     <t>24,051,199</t>
   </si>
   <si>
-    <t>90年/110歲</t>
-  </si>
-  <si>
     <t>25,614,527</t>
   </si>
   <si>
-    <t>91年/111歲</t>
-  </si>
-  <si>
     <t>27,279,471</t>
   </si>
   <si>
-    <t>92年/112歲</t>
-  </si>
-  <si>
     <t>29,052,637</t>
   </si>
   <si>
-    <t>93年/113歲</t>
-  </si>
-  <si>
     <t>30,941,058</t>
   </si>
   <si>
-    <t>94年/114歲</t>
-  </si>
-  <si>
     <t>32,952,227</t>
   </si>
   <si>
-    <t>95年/115歲</t>
-  </si>
-  <si>
     <t>35,094,122</t>
   </si>
   <si>
-    <t>96年/116歲</t>
-  </si>
-  <si>
     <t>37,375,240</t>
   </si>
   <si>
-    <t>97年/117歲</t>
-  </si>
-  <si>
     <t>39,804,630</t>
   </si>
   <si>
-    <t>98年/118歲</t>
-  </si>
-  <si>
     <t>42,391,931</t>
   </si>
   <si>
-    <t>99年/119歲</t>
-  </si>
-  <si>
     <t>45,147,407</t>
-  </si>
-  <si>
-    <t>100年/120歲</t>
   </si>
   <si>
     <t>48,081,988</t>
@@ -627,6 +327,308 @@
   <si>
     <t>此模板为不提取时计算用模板，请将保单对应预期保单价值拷贝进E列即可</t>
     <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>1年</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>2年</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>3年</t>
+  </si>
+  <si>
+    <t>4年</t>
+  </si>
+  <si>
+    <t>5年</t>
+  </si>
+  <si>
+    <t>6年</t>
+  </si>
+  <si>
+    <t>7年</t>
+  </si>
+  <si>
+    <t>8年</t>
+  </si>
+  <si>
+    <t>9年</t>
+  </si>
+  <si>
+    <t>10年</t>
+  </si>
+  <si>
+    <t>11年</t>
+  </si>
+  <si>
+    <t>12年</t>
+  </si>
+  <si>
+    <t>13年</t>
+  </si>
+  <si>
+    <t>14年</t>
+  </si>
+  <si>
+    <t>15年</t>
+  </si>
+  <si>
+    <t>16年</t>
+  </si>
+  <si>
+    <t>17年</t>
+  </si>
+  <si>
+    <t>18年</t>
+  </si>
+  <si>
+    <t>19年</t>
+  </si>
+  <si>
+    <t>20年</t>
+  </si>
+  <si>
+    <t>21年</t>
+  </si>
+  <si>
+    <t>22年</t>
+  </si>
+  <si>
+    <t>23年</t>
+  </si>
+  <si>
+    <t>24年</t>
+  </si>
+  <si>
+    <t>25年</t>
+  </si>
+  <si>
+    <t>26年</t>
+  </si>
+  <si>
+    <t>27年</t>
+  </si>
+  <si>
+    <t>28年</t>
+  </si>
+  <si>
+    <t>29年</t>
+  </si>
+  <si>
+    <t>30年</t>
+  </si>
+  <si>
+    <t>31年</t>
+  </si>
+  <si>
+    <t>32年</t>
+  </si>
+  <si>
+    <t>33年</t>
+  </si>
+  <si>
+    <t>34年</t>
+  </si>
+  <si>
+    <t>35年</t>
+  </si>
+  <si>
+    <t>36年</t>
+  </si>
+  <si>
+    <t>37年</t>
+  </si>
+  <si>
+    <t>38年</t>
+  </si>
+  <si>
+    <t>39年</t>
+  </si>
+  <si>
+    <t>40年</t>
+  </si>
+  <si>
+    <t>41年</t>
+  </si>
+  <si>
+    <t>42年</t>
+  </si>
+  <si>
+    <t>43年</t>
+  </si>
+  <si>
+    <t>44年</t>
+  </si>
+  <si>
+    <t>45年</t>
+  </si>
+  <si>
+    <t>46年</t>
+  </si>
+  <si>
+    <t>47年</t>
+  </si>
+  <si>
+    <t>48年</t>
+  </si>
+  <si>
+    <t>49年</t>
+  </si>
+  <si>
+    <t>50年</t>
+  </si>
+  <si>
+    <t>51年</t>
+  </si>
+  <si>
+    <t>52年</t>
+  </si>
+  <si>
+    <t>53年</t>
+  </si>
+  <si>
+    <t>54年</t>
+  </si>
+  <si>
+    <t>55年</t>
+  </si>
+  <si>
+    <t>56年</t>
+  </si>
+  <si>
+    <t>57年</t>
+  </si>
+  <si>
+    <t>58年</t>
+  </si>
+  <si>
+    <t>59年</t>
+  </si>
+  <si>
+    <t>60年</t>
+  </si>
+  <si>
+    <t>61年</t>
+  </si>
+  <si>
+    <t>62年</t>
+  </si>
+  <si>
+    <t>63年</t>
+  </si>
+  <si>
+    <t>64年</t>
+  </si>
+  <si>
+    <t>65年</t>
+  </si>
+  <si>
+    <t>66年</t>
+  </si>
+  <si>
+    <t>67年</t>
+  </si>
+  <si>
+    <t>68年</t>
+  </si>
+  <si>
+    <t>69年</t>
+  </si>
+  <si>
+    <t>70年</t>
+  </si>
+  <si>
+    <t>71年</t>
+  </si>
+  <si>
+    <t>72年</t>
+  </si>
+  <si>
+    <t>73年</t>
+  </si>
+  <si>
+    <t>74年</t>
+  </si>
+  <si>
+    <t>75年</t>
+  </si>
+  <si>
+    <t>76年</t>
+  </si>
+  <si>
+    <t>77年</t>
+  </si>
+  <si>
+    <t>78年</t>
+  </si>
+  <si>
+    <t>79年</t>
+  </si>
+  <si>
+    <t>80年</t>
+  </si>
+  <si>
+    <t>81年</t>
+  </si>
+  <si>
+    <t>82年</t>
+  </si>
+  <si>
+    <t>83年</t>
+  </si>
+  <si>
+    <t>84年</t>
+  </si>
+  <si>
+    <t>85年</t>
+  </si>
+  <si>
+    <t>86年</t>
+  </si>
+  <si>
+    <t>87年</t>
+  </si>
+  <si>
+    <t>88年</t>
+  </si>
+  <si>
+    <t>89年</t>
+  </si>
+  <si>
+    <t>90年</t>
+  </si>
+  <si>
+    <t>91年</t>
+  </si>
+  <si>
+    <t>92年</t>
+  </si>
+  <si>
+    <t>93年</t>
+  </si>
+  <si>
+    <t>94年</t>
+  </si>
+  <si>
+    <t>95年</t>
+  </si>
+  <si>
+    <t>96年</t>
+  </si>
+  <si>
+    <t>97年</t>
+  </si>
+  <si>
+    <t>98年</t>
+  </si>
+  <si>
+    <t>99年</t>
+  </si>
+  <si>
+    <t>100年</t>
   </si>
 </sst>
 </file>
@@ -1119,7 +1121,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>201</v>
+        <v>101</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -1147,7 +1149,7 @@
     </row>
     <row r="3" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1160,13 +1162,13 @@
     </row>
     <row r="4" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>103</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -1175,13 +1177,13 @@
     </row>
     <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>104</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
@@ -1190,13 +1192,13 @@
     </row>
     <row r="6" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>7</v>
+        <v>105</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
@@ -1205,13 +1207,13 @@
     </row>
     <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>9</v>
+        <v>106</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
@@ -1220,13 +1222,13 @@
     </row>
     <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>11</v>
+        <v>107</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -1234,14 +1236,14 @@
       <c r="I8" s="1"/>
     </row>
     <row r="9" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>13</v>
+      <c r="A9" s="1" t="s">
+        <v>108</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -1249,14 +1251,14 @@
       <c r="I9" s="2"/>
     </row>
     <row r="10" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>15</v>
+      <c r="A10" s="1" t="s">
+        <v>109</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
@@ -1264,14 +1266,14 @@
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>17</v>
+      <c r="A11" s="1" t="s">
+        <v>110</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -1279,14 +1281,14 @@
       <c r="I11" s="2"/>
     </row>
     <row r="12" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>19</v>
+      <c r="A12" s="1" t="s">
+        <v>111</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
@@ -1294,14 +1296,14 @@
       <c r="I12" s="2"/>
     </row>
     <row r="13" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>21</v>
+      <c r="A13" s="1" t="s">
+        <v>112</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
@@ -1309,14 +1311,14 @@
       <c r="I13" s="2"/>
     </row>
     <row r="14" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
-        <v>23</v>
+      <c r="A14" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
@@ -1324,14 +1326,14 @@
       <c r="I14" s="2"/>
     </row>
     <row r="15" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
-        <v>25</v>
+      <c r="A15" s="1" t="s">
+        <v>114</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
@@ -1339,14 +1341,14 @@
       <c r="I15" s="2"/>
     </row>
     <row r="16" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
-        <v>27</v>
+      <c r="A16" s="1" t="s">
+        <v>115</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
@@ -1354,14 +1356,14 @@
       <c r="I16" s="2"/>
     </row>
     <row r="17" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
-        <v>29</v>
+      <c r="A17" s="1" t="s">
+        <v>116</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -1369,14 +1371,14 @@
       <c r="I17" s="2"/>
     </row>
     <row r="18" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>31</v>
+      <c r="A18" s="1" t="s">
+        <v>117</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -1384,14 +1386,14 @@
       <c r="I18" s="2"/>
     </row>
     <row r="19" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
-        <v>33</v>
+      <c r="A19" s="1" t="s">
+        <v>118</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
@@ -1399,14 +1401,14 @@
       <c r="I19" s="2"/>
     </row>
     <row r="20" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="2" t="s">
-        <v>35</v>
+      <c r="A20" s="1" t="s">
+        <v>119</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -1414,14 +1416,14 @@
       <c r="I20" s="2"/>
     </row>
     <row r="21" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
-        <v>37</v>
+      <c r="A21" s="1" t="s">
+        <v>120</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -1429,14 +1431,14 @@
       <c r="I21" s="2"/>
     </row>
     <row r="22" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
-        <v>39</v>
+      <c r="A22" s="1" t="s">
+        <v>121</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -1444,14 +1446,14 @@
       <c r="I22" s="2"/>
     </row>
     <row r="23" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
-        <v>41</v>
+      <c r="A23" s="1" t="s">
+        <v>122</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
@@ -1459,14 +1461,14 @@
       <c r="I23" s="2"/>
     </row>
     <row r="24" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
-        <v>43</v>
+      <c r="A24" s="1" t="s">
+        <v>123</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
@@ -1474,14 +1476,14 @@
       <c r="I24" s="2"/>
     </row>
     <row r="25" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
-        <v>45</v>
+      <c r="A25" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -1489,14 +1491,14 @@
       <c r="I25" s="2"/>
     </row>
     <row r="26" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="2" t="s">
-        <v>47</v>
+      <c r="A26" s="1" t="s">
+        <v>125</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2" t="s">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -1504,14 +1506,14 @@
       <c r="I26" s="2"/>
     </row>
     <row r="27" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="2" t="s">
-        <v>49</v>
+      <c r="A27" s="1" t="s">
+        <v>126</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -1519,14 +1521,14 @@
       <c r="I27" s="2"/>
     </row>
     <row r="28" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="2" t="s">
-        <v>51</v>
+      <c r="A28" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2" t="s">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -1534,14 +1536,14 @@
       <c r="I28" s="2"/>
     </row>
     <row r="29" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="2" t="s">
-        <v>53</v>
+      <c r="A29" s="1" t="s">
+        <v>128</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2" t="s">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
@@ -1549,14 +1551,14 @@
       <c r="I29" s="2"/>
     </row>
     <row r="30" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
-        <v>55</v>
+      <c r="A30" s="1" t="s">
+        <v>129</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
@@ -1564,14 +1566,14 @@
       <c r="I30" s="2"/>
     </row>
     <row r="31" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="2" t="s">
-        <v>57</v>
+      <c r="A31" s="1" t="s">
+        <v>130</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
@@ -1579,14 +1581,14 @@
       <c r="I31" s="2"/>
     </row>
     <row r="32" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="2" t="s">
-        <v>59</v>
+      <c r="A32" s="1" t="s">
+        <v>131</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2" t="s">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
@@ -1594,14 +1596,14 @@
       <c r="I32" s="2"/>
     </row>
     <row r="33" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="2" t="s">
-        <v>61</v>
+      <c r="A33" s="1" t="s">
+        <v>132</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
@@ -1609,14 +1611,14 @@
       <c r="I33" s="2"/>
     </row>
     <row r="34" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="2" t="s">
-        <v>63</v>
+      <c r="A34" s="1" t="s">
+        <v>133</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2" t="s">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
@@ -1624,14 +1626,14 @@
       <c r="I34" s="2"/>
     </row>
     <row r="35" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="2" t="s">
-        <v>65</v>
+      <c r="A35" s="1" t="s">
+        <v>134</v>
       </c>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2" t="s">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
@@ -1639,14 +1641,14 @@
       <c r="I35" s="2"/>
     </row>
     <row r="36" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="2" t="s">
-        <v>67</v>
+      <c r="A36" s="1" t="s">
+        <v>135</v>
       </c>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2" t="s">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
@@ -1654,14 +1656,14 @@
       <c r="I36" s="2"/>
     </row>
     <row r="37" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="2" t="s">
-        <v>69</v>
+      <c r="A37" s="1" t="s">
+        <v>136</v>
       </c>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
@@ -1669,14 +1671,14 @@
       <c r="I37" s="2"/>
     </row>
     <row r="38" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="2" t="s">
-        <v>71</v>
+      <c r="A38" s="1" t="s">
+        <v>137</v>
       </c>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2" t="s">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
@@ -1684,14 +1686,14 @@
       <c r="I38" s="2"/>
     </row>
     <row r="39" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="2" t="s">
-        <v>73</v>
+      <c r="A39" s="1" t="s">
+        <v>138</v>
       </c>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2" t="s">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
@@ -1699,14 +1701,14 @@
       <c r="I39" s="2"/>
     </row>
     <row r="40" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="2" t="s">
-        <v>75</v>
+      <c r="A40" s="1" t="s">
+        <v>139</v>
       </c>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
@@ -1714,14 +1716,14 @@
       <c r="I40" s="2"/>
     </row>
     <row r="41" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="2" t="s">
-        <v>77</v>
+      <c r="A41" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
@@ -1729,14 +1731,14 @@
       <c r="I41" s="2"/>
     </row>
     <row r="42" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="2" t="s">
-        <v>79</v>
+      <c r="A42" s="1" t="s">
+        <v>141</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2" t="s">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
@@ -1744,14 +1746,14 @@
       <c r="I42" s="2"/>
     </row>
     <row r="43" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="2" t="s">
-        <v>81</v>
+      <c r="A43" s="1" t="s">
+        <v>142</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2" t="s">
-        <v>82</v>
+        <v>41</v>
       </c>
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
@@ -1759,14 +1761,14 @@
       <c r="I43" s="2"/>
     </row>
     <row r="44" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="2" t="s">
-        <v>83</v>
+      <c r="A44" s="1" t="s">
+        <v>143</v>
       </c>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2" t="s">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
@@ -1774,14 +1776,14 @@
       <c r="I44" s="2"/>
     </row>
     <row r="45" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="2" t="s">
-        <v>85</v>
+      <c r="A45" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2" t="s">
-        <v>86</v>
+        <v>43</v>
       </c>
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
@@ -1789,14 +1791,14 @@
       <c r="I45" s="2"/>
     </row>
     <row r="46" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="2" t="s">
-        <v>87</v>
+      <c r="A46" s="1" t="s">
+        <v>145</v>
       </c>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="2" t="s">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
@@ -1804,14 +1806,14 @@
       <c r="I46" s="2"/>
     </row>
     <row r="47" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="2" t="s">
-        <v>89</v>
+      <c r="A47" s="1" t="s">
+        <v>146</v>
       </c>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="F47" s="2"/>
       <c r="G47" s="2"/>
@@ -1819,14 +1821,14 @@
       <c r="I47" s="2"/>
     </row>
     <row r="48" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="2" t="s">
-        <v>91</v>
+      <c r="A48" s="1" t="s">
+        <v>147</v>
       </c>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="2" t="s">
-        <v>92</v>
+        <v>46</v>
       </c>
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
@@ -1834,14 +1836,14 @@
       <c r="I48" s="2"/>
     </row>
     <row r="49" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="2" t="s">
-        <v>93</v>
+      <c r="A49" s="1" t="s">
+        <v>148</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2" t="s">
-        <v>94</v>
+        <v>47</v>
       </c>
       <c r="F49" s="2"/>
       <c r="G49" s="2"/>
@@ -1849,14 +1851,14 @@
       <c r="I49" s="2"/>
     </row>
     <row r="50" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="2" t="s">
-        <v>95</v>
+      <c r="A50" s="1" t="s">
+        <v>149</v>
       </c>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
       <c r="E50" s="2" t="s">
-        <v>96</v>
+        <v>48</v>
       </c>
       <c r="F50" s="2"/>
       <c r="G50" s="2"/>
@@ -1864,14 +1866,14 @@
       <c r="I50" s="2"/>
     </row>
     <row r="51" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="2" t="s">
-        <v>97</v>
+      <c r="A51" s="1" t="s">
+        <v>150</v>
       </c>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="E51" s="2" t="s">
-        <v>98</v>
+        <v>49</v>
       </c>
       <c r="F51" s="2"/>
       <c r="G51" s="2"/>
@@ -1879,14 +1881,14 @@
       <c r="I51" s="2"/>
     </row>
     <row r="52" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="2" t="s">
-        <v>99</v>
+      <c r="A52" s="1" t="s">
+        <v>151</v>
       </c>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="E52" s="2" t="s">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
@@ -1894,14 +1896,14 @@
       <c r="I52" s="2"/>
     </row>
     <row r="53" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="2" t="s">
-        <v>101</v>
+      <c r="A53" s="1" t="s">
+        <v>152</v>
       </c>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F53" s="2"/>
       <c r="G53" s="2"/>
@@ -1909,14 +1911,14 @@
       <c r="I53" s="2"/>
     </row>
     <row r="54" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="2" t="s">
-        <v>103</v>
+      <c r="A54" s="1" t="s">
+        <v>153</v>
       </c>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="2" t="s">
-        <v>104</v>
+        <v>52</v>
       </c>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
@@ -1924,14 +1926,14 @@
       <c r="I54" s="2"/>
     </row>
     <row r="55" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="2" t="s">
-        <v>105</v>
+      <c r="A55" s="1" t="s">
+        <v>154</v>
       </c>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
       <c r="E55" s="2" t="s">
-        <v>106</v>
+        <v>53</v>
       </c>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
@@ -1939,14 +1941,14 @@
       <c r="I55" s="2"/>
     </row>
     <row r="56" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="2" t="s">
-        <v>107</v>
+      <c r="A56" s="1" t="s">
+        <v>155</v>
       </c>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
       <c r="E56" s="2" t="s">
-        <v>108</v>
+        <v>54</v>
       </c>
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
@@ -1954,14 +1956,14 @@
       <c r="I56" s="2"/>
     </row>
     <row r="57" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="2" t="s">
-        <v>109</v>
+      <c r="A57" s="1" t="s">
+        <v>156</v>
       </c>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2" t="s">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="F57" s="2"/>
       <c r="G57" s="2"/>
@@ -1969,14 +1971,14 @@
       <c r="I57" s="2"/>
     </row>
     <row r="58" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="2" t="s">
-        <v>111</v>
+      <c r="A58" s="1" t="s">
+        <v>157</v>
       </c>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
       <c r="E58" s="2" t="s">
-        <v>112</v>
+        <v>56</v>
       </c>
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
@@ -1984,14 +1986,14 @@
       <c r="I58" s="2"/>
     </row>
     <row r="59" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="2" t="s">
-        <v>113</v>
+      <c r="A59" s="1" t="s">
+        <v>158</v>
       </c>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
       <c r="E59" s="2" t="s">
-        <v>114</v>
+        <v>57</v>
       </c>
       <c r="F59" s="2"/>
       <c r="G59" s="2"/>
@@ -1999,14 +2001,14 @@
       <c r="I59" s="2"/>
     </row>
     <row r="60" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="2" t="s">
-        <v>115</v>
+      <c r="A60" s="1" t="s">
+        <v>159</v>
       </c>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
       <c r="E60" s="2" t="s">
-        <v>116</v>
+        <v>58</v>
       </c>
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
@@ -2014,14 +2016,14 @@
       <c r="I60" s="2"/>
     </row>
     <row r="61" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="2" t="s">
-        <v>117</v>
+      <c r="A61" s="1" t="s">
+        <v>160</v>
       </c>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
       <c r="E61" s="2" t="s">
-        <v>118</v>
+        <v>59</v>
       </c>
       <c r="F61" s="2"/>
       <c r="G61" s="2"/>
@@ -2029,14 +2031,14 @@
       <c r="I61" s="2"/>
     </row>
     <row r="62" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="2" t="s">
-        <v>119</v>
+      <c r="A62" s="1" t="s">
+        <v>161</v>
       </c>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
       <c r="E62" s="2" t="s">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
@@ -2044,14 +2046,14 @@
       <c r="I62" s="2"/>
     </row>
     <row r="63" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="2" t="s">
-        <v>121</v>
+      <c r="A63" s="1" t="s">
+        <v>162</v>
       </c>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
       <c r="E63" s="2" t="s">
-        <v>122</v>
+        <v>61</v>
       </c>
       <c r="F63" s="2"/>
       <c r="G63" s="2"/>
@@ -2059,14 +2061,14 @@
       <c r="I63" s="2"/>
     </row>
     <row r="64" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="2" t="s">
-        <v>123</v>
+      <c r="A64" s="1" t="s">
+        <v>163</v>
       </c>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
       <c r="E64" s="2" t="s">
-        <v>124</v>
+        <v>62</v>
       </c>
       <c r="F64" s="2"/>
       <c r="G64" s="2"/>
@@ -2074,14 +2076,14 @@
       <c r="I64" s="2"/>
     </row>
     <row r="65" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="2" t="s">
-        <v>125</v>
+      <c r="A65" s="1" t="s">
+        <v>164</v>
       </c>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
       <c r="E65" s="2" t="s">
-        <v>126</v>
+        <v>63</v>
       </c>
       <c r="F65" s="2"/>
       <c r="G65" s="2"/>
@@ -2089,14 +2091,14 @@
       <c r="I65" s="2"/>
     </row>
     <row r="66" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A66" s="2" t="s">
-        <v>127</v>
+      <c r="A66" s="1" t="s">
+        <v>165</v>
       </c>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
       <c r="E66" s="2" t="s">
-        <v>128</v>
+        <v>64</v>
       </c>
       <c r="F66" s="2"/>
       <c r="G66" s="2"/>
@@ -2104,14 +2106,14 @@
       <c r="I66" s="2"/>
     </row>
     <row r="67" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="2" t="s">
-        <v>129</v>
+      <c r="A67" s="1" t="s">
+        <v>166</v>
       </c>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
       <c r="E67" s="2" t="s">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="F67" s="2"/>
       <c r="G67" s="2"/>
@@ -2119,14 +2121,14 @@
       <c r="I67" s="2"/>
     </row>
     <row r="68" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="2" t="s">
-        <v>131</v>
+      <c r="A68" s="1" t="s">
+        <v>167</v>
       </c>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
       <c r="D68" s="2"/>
       <c r="E68" s="2" t="s">
-        <v>132</v>
+        <v>66</v>
       </c>
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
@@ -2134,14 +2136,14 @@
       <c r="I68" s="2"/>
     </row>
     <row r="69" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="2" t="s">
-        <v>133</v>
+      <c r="A69" s="1" t="s">
+        <v>168</v>
       </c>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
       <c r="D69" s="2"/>
       <c r="E69" s="2" t="s">
-        <v>134</v>
+        <v>67</v>
       </c>
       <c r="F69" s="2"/>
       <c r="G69" s="2"/>
@@ -2149,14 +2151,14 @@
       <c r="I69" s="2"/>
     </row>
     <row r="70" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="2" t="s">
-        <v>135</v>
+      <c r="A70" s="1" t="s">
+        <v>169</v>
       </c>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
       <c r="D70" s="2"/>
       <c r="E70" s="2" t="s">
-        <v>136</v>
+        <v>68</v>
       </c>
       <c r="F70" s="2"/>
       <c r="G70" s="2"/>
@@ -2164,14 +2166,14 @@
       <c r="I70" s="2"/>
     </row>
     <row r="71" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="2" t="s">
-        <v>137</v>
+      <c r="A71" s="1" t="s">
+        <v>170</v>
       </c>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
       <c r="D71" s="2"/>
       <c r="E71" s="2" t="s">
-        <v>138</v>
+        <v>69</v>
       </c>
       <c r="F71" s="2"/>
       <c r="G71" s="2"/>
@@ -2179,14 +2181,14 @@
       <c r="I71" s="2"/>
     </row>
     <row r="72" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="2" t="s">
-        <v>139</v>
+      <c r="A72" s="1" t="s">
+        <v>171</v>
       </c>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
       <c r="D72" s="2"/>
       <c r="E72" s="2" t="s">
-        <v>140</v>
+        <v>70</v>
       </c>
       <c r="F72" s="2"/>
       <c r="G72" s="2"/>
@@ -2194,14 +2196,14 @@
       <c r="I72" s="2"/>
     </row>
     <row r="73" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A73" s="2" t="s">
-        <v>141</v>
+      <c r="A73" s="1" t="s">
+        <v>172</v>
       </c>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
       <c r="D73" s="2"/>
       <c r="E73" s="2" t="s">
-        <v>142</v>
+        <v>71</v>
       </c>
       <c r="F73" s="2"/>
       <c r="G73" s="2"/>
@@ -2209,14 +2211,14 @@
       <c r="I73" s="2"/>
     </row>
     <row r="74" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A74" s="2" t="s">
-        <v>143</v>
+      <c r="A74" s="1" t="s">
+        <v>173</v>
       </c>
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
       <c r="D74" s="2"/>
       <c r="E74" s="2" t="s">
-        <v>144</v>
+        <v>72</v>
       </c>
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
@@ -2224,14 +2226,14 @@
       <c r="I74" s="2"/>
     </row>
     <row r="75" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A75" s="2" t="s">
-        <v>145</v>
+      <c r="A75" s="1" t="s">
+        <v>174</v>
       </c>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
       <c r="D75" s="2"/>
       <c r="E75" s="2" t="s">
-        <v>146</v>
+        <v>73</v>
       </c>
       <c r="F75" s="2"/>
       <c r="G75" s="2"/>
@@ -2239,14 +2241,14 @@
       <c r="I75" s="2"/>
     </row>
     <row r="76" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="2" t="s">
-        <v>147</v>
+      <c r="A76" s="1" t="s">
+        <v>175</v>
       </c>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
       <c r="D76" s="2"/>
       <c r="E76" s="2" t="s">
-        <v>148</v>
+        <v>74</v>
       </c>
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
@@ -2254,14 +2256,14 @@
       <c r="I76" s="2"/>
     </row>
     <row r="77" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="2" t="s">
-        <v>149</v>
+      <c r="A77" s="1" t="s">
+        <v>176</v>
       </c>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
       <c r="D77" s="2"/>
       <c r="E77" s="2" t="s">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="F77" s="2"/>
       <c r="G77" s="2"/>
@@ -2269,14 +2271,14 @@
       <c r="I77" s="2"/>
     </row>
     <row r="78" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="2" t="s">
-        <v>151</v>
+      <c r="A78" s="1" t="s">
+        <v>177</v>
       </c>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
       <c r="E78" s="2" t="s">
-        <v>152</v>
+        <v>76</v>
       </c>
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
@@ -2284,14 +2286,14 @@
       <c r="I78" s="2"/>
     </row>
     <row r="79" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="2" t="s">
-        <v>153</v>
+      <c r="A79" s="1" t="s">
+        <v>178</v>
       </c>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
       <c r="E79" s="2" t="s">
-        <v>154</v>
+        <v>77</v>
       </c>
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
@@ -2299,14 +2301,14 @@
       <c r="I79" s="2"/>
     </row>
     <row r="80" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A80" s="2" t="s">
-        <v>155</v>
+      <c r="A80" s="1" t="s">
+        <v>179</v>
       </c>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
       <c r="E80" s="2" t="s">
-        <v>156</v>
+        <v>78</v>
       </c>
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
@@ -2314,14 +2316,14 @@
       <c r="I80" s="2"/>
     </row>
     <row r="81" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A81" s="2" t="s">
-        <v>157</v>
+      <c r="A81" s="1" t="s">
+        <v>180</v>
       </c>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
       <c r="D81" s="2"/>
       <c r="E81" s="2" t="s">
-        <v>158</v>
+        <v>79</v>
       </c>
       <c r="F81" s="2"/>
       <c r="G81" s="2"/>
@@ -2329,14 +2331,14 @@
       <c r="I81" s="2"/>
     </row>
     <row r="82" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A82" s="2" t="s">
-        <v>159</v>
+      <c r="A82" s="1" t="s">
+        <v>181</v>
       </c>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
       <c r="D82" s="2"/>
       <c r="E82" s="2" t="s">
-        <v>160</v>
+        <v>80</v>
       </c>
       <c r="F82" s="2"/>
       <c r="G82" s="2"/>
@@ -2344,14 +2346,14 @@
       <c r="I82" s="2"/>
     </row>
     <row r="83" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A83" s="2" t="s">
-        <v>161</v>
+      <c r="A83" s="1" t="s">
+        <v>182</v>
       </c>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
       <c r="D83" s="2"/>
       <c r="E83" s="2" t="s">
-        <v>162</v>
+        <v>81</v>
       </c>
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
@@ -2359,14 +2361,14 @@
       <c r="I83" s="2"/>
     </row>
     <row r="84" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A84" s="2" t="s">
-        <v>163</v>
+      <c r="A84" s="1" t="s">
+        <v>183</v>
       </c>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
       <c r="D84" s="2"/>
       <c r="E84" s="2" t="s">
-        <v>164</v>
+        <v>82</v>
       </c>
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>
@@ -2374,14 +2376,14 @@
       <c r="I84" s="2"/>
     </row>
     <row r="85" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A85" s="2" t="s">
-        <v>165</v>
+      <c r="A85" s="1" t="s">
+        <v>184</v>
       </c>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
       <c r="D85" s="2"/>
       <c r="E85" s="2" t="s">
-        <v>166</v>
+        <v>83</v>
       </c>
       <c r="F85" s="2"/>
       <c r="G85" s="2"/>
@@ -2389,14 +2391,14 @@
       <c r="I85" s="2"/>
     </row>
     <row r="86" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A86" s="2" t="s">
-        <v>167</v>
+      <c r="A86" s="1" t="s">
+        <v>185</v>
       </c>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
       <c r="E86" s="2" t="s">
-        <v>168</v>
+        <v>84</v>
       </c>
       <c r="F86" s="2"/>
       <c r="G86" s="2"/>
@@ -2404,14 +2406,14 @@
       <c r="I86" s="2"/>
     </row>
     <row r="87" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A87" s="2" t="s">
-        <v>169</v>
+      <c r="A87" s="1" t="s">
+        <v>186</v>
       </c>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
       <c r="E87" s="2" t="s">
-        <v>170</v>
+        <v>85</v>
       </c>
       <c r="F87" s="2"/>
       <c r="G87" s="2"/>
@@ -2419,14 +2421,14 @@
       <c r="I87" s="2"/>
     </row>
     <row r="88" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A88" s="2" t="s">
-        <v>171</v>
+      <c r="A88" s="1" t="s">
+        <v>187</v>
       </c>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
       <c r="E88" s="2" t="s">
-        <v>172</v>
+        <v>86</v>
       </c>
       <c r="F88" s="2"/>
       <c r="G88" s="2"/>
@@ -2434,14 +2436,14 @@
       <c r="I88" s="2"/>
     </row>
     <row r="89" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A89" s="2" t="s">
-        <v>173</v>
+      <c r="A89" s="1" t="s">
+        <v>188</v>
       </c>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
       <c r="D89" s="2"/>
       <c r="E89" s="2" t="s">
-        <v>174</v>
+        <v>87</v>
       </c>
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
@@ -2449,14 +2451,14 @@
       <c r="I89" s="2"/>
     </row>
     <row r="90" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A90" s="2" t="s">
-        <v>175</v>
+      <c r="A90" s="1" t="s">
+        <v>189</v>
       </c>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
       <c r="E90" s="2" t="s">
-        <v>176</v>
+        <v>88</v>
       </c>
       <c r="F90" s="2"/>
       <c r="G90" s="2"/>
@@ -2464,14 +2466,14 @@
       <c r="I90" s="2"/>
     </row>
     <row r="91" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A91" s="2" t="s">
-        <v>177</v>
+      <c r="A91" s="1" t="s">
+        <v>190</v>
       </c>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
       <c r="D91" s="2"/>
       <c r="E91" s="2" t="s">
-        <v>178</v>
+        <v>89</v>
       </c>
       <c r="F91" s="2"/>
       <c r="G91" s="2"/>
@@ -2479,14 +2481,14 @@
       <c r="I91" s="2"/>
     </row>
     <row r="92" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A92" s="2" t="s">
-        <v>179</v>
+      <c r="A92" s="1" t="s">
+        <v>191</v>
       </c>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
       <c r="D92" s="2"/>
       <c r="E92" s="2" t="s">
-        <v>180</v>
+        <v>90</v>
       </c>
       <c r="F92" s="2"/>
       <c r="G92" s="2"/>
@@ -2494,14 +2496,14 @@
       <c r="I92" s="2"/>
     </row>
     <row r="93" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A93" s="2" t="s">
-        <v>181</v>
+      <c r="A93" s="1" t="s">
+        <v>192</v>
       </c>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
       <c r="D93" s="2"/>
       <c r="E93" s="2" t="s">
-        <v>182</v>
+        <v>91</v>
       </c>
       <c r="F93" s="2"/>
       <c r="G93" s="2"/>
@@ -2509,14 +2511,14 @@
       <c r="I93" s="2"/>
     </row>
     <row r="94" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A94" s="2" t="s">
-        <v>183</v>
+      <c r="A94" s="1" t="s">
+        <v>193</v>
       </c>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
       <c r="D94" s="2"/>
       <c r="E94" s="2" t="s">
-        <v>184</v>
+        <v>92</v>
       </c>
       <c r="F94" s="2"/>
       <c r="G94" s="2"/>
@@ -2524,14 +2526,14 @@
       <c r="I94" s="2"/>
     </row>
     <row r="95" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A95" s="2" t="s">
-        <v>185</v>
+      <c r="A95" s="1" t="s">
+        <v>194</v>
       </c>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
       <c r="D95" s="2"/>
       <c r="E95" s="2" t="s">
-        <v>186</v>
+        <v>93</v>
       </c>
       <c r="F95" s="2"/>
       <c r="G95" s="2"/>
@@ -2539,14 +2541,14 @@
       <c r="I95" s="2"/>
     </row>
     <row r="96" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A96" s="2" t="s">
-        <v>187</v>
+      <c r="A96" s="1" t="s">
+        <v>195</v>
       </c>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
       <c r="D96" s="2"/>
       <c r="E96" s="2" t="s">
-        <v>188</v>
+        <v>94</v>
       </c>
       <c r="F96" s="2"/>
       <c r="G96" s="2"/>
@@ -2554,14 +2556,14 @@
       <c r="I96" s="2"/>
     </row>
     <row r="97" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A97" s="2" t="s">
-        <v>189</v>
+      <c r="A97" s="1" t="s">
+        <v>196</v>
       </c>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
       <c r="D97" s="2"/>
       <c r="E97" s="2" t="s">
-        <v>190</v>
+        <v>95</v>
       </c>
       <c r="F97" s="2"/>
       <c r="G97" s="2"/>
@@ -2569,14 +2571,14 @@
       <c r="I97" s="2"/>
     </row>
     <row r="98" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A98" s="2" t="s">
-        <v>191</v>
+      <c r="A98" s="1" t="s">
+        <v>197</v>
       </c>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
       <c r="D98" s="2"/>
       <c r="E98" s="2" t="s">
-        <v>192</v>
+        <v>96</v>
       </c>
       <c r="F98" s="2"/>
       <c r="G98" s="2"/>
@@ -2584,14 +2586,14 @@
       <c r="I98" s="2"/>
     </row>
     <row r="99" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A99" s="2" t="s">
-        <v>193</v>
+      <c r="A99" s="1" t="s">
+        <v>198</v>
       </c>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
       <c r="D99" s="2"/>
       <c r="E99" s="2" t="s">
-        <v>194</v>
+        <v>97</v>
       </c>
       <c r="F99" s="2"/>
       <c r="G99" s="2"/>
@@ -2599,14 +2601,14 @@
       <c r="I99" s="2"/>
     </row>
     <row r="100" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A100" s="2" t="s">
-        <v>195</v>
+      <c r="A100" s="1" t="s">
+        <v>199</v>
       </c>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
       <c r="D100" s="2"/>
       <c r="E100" s="2" t="s">
-        <v>196</v>
+        <v>98</v>
       </c>
       <c r="F100" s="2"/>
       <c r="G100" s="2"/>
@@ -2614,14 +2616,14 @@
       <c r="I100" s="2"/>
     </row>
     <row r="101" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A101" s="2" t="s">
-        <v>197</v>
+      <c r="A101" s="1" t="s">
+        <v>200</v>
       </c>
       <c r="B101" s="2"/>
       <c r="C101" s="2"/>
       <c r="D101" s="2"/>
       <c r="E101" s="2" t="s">
-        <v>198</v>
+        <v>99</v>
       </c>
       <c r="F101" s="2"/>
       <c r="G101" s="2"/>
@@ -2629,14 +2631,14 @@
       <c r="I101" s="2"/>
     </row>
     <row r="102" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A102" s="2" t="s">
-        <v>199</v>
+      <c r="A102" s="1" t="s">
+        <v>201</v>
       </c>
       <c r="B102" s="2"/>
       <c r="C102" s="2"/>
       <c r="D102" s="2"/>
       <c r="E102" s="2" t="s">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F102" s="2"/>
       <c r="G102" s="2"/>

</xml_diff>